<commit_message>
update to version 3
</commit_message>
<xml_diff>
--- a/requirements_file/markers_brain.xlsx
+++ b/requirements_file/markers_brain.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\merag\Git\JSEQ_scRNAseq\requirements_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A408A0F-FC7B-4BAC-BEFB-32CCD47526CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E90976-04C8-402C-9D29-AA28847A5865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="class" sheetId="1" r:id="rId1"/>
@@ -46,12 +46,6 @@
     <t>Microglial</t>
   </si>
   <si>
-    <t>Astrocytes</t>
-  </si>
-  <si>
-    <t>Oligodendrocytes</t>
-  </si>
-  <si>
     <t>+AQP4</t>
   </si>
   <si>
@@ -178,9 +172,6 @@
     <t>FOXJ1</t>
   </si>
   <si>
-    <t>Macrophages</t>
-  </si>
-  <si>
     <t>+NOS1</t>
   </si>
   <si>
@@ -196,9 +187,6 @@
     <t>VTN</t>
   </si>
   <si>
-    <t>Pericytes</t>
-  </si>
-  <si>
     <t>+VTN</t>
   </si>
   <si>
@@ -223,12 +211,6 @@
     <t>+SLC5A8</t>
   </si>
   <si>
-    <t>Purkinji</t>
-  </si>
-  <si>
-    <t>Tanacytes</t>
-  </si>
-  <si>
     <t>+CSPG4</t>
   </si>
   <si>
@@ -334,12 +316,6 @@
     <t>MUSTN1</t>
   </si>
   <si>
-    <t>NPCs</t>
-  </si>
-  <si>
-    <t>GPCs</t>
-  </si>
-  <si>
     <t>GBX2</t>
   </si>
   <si>
@@ -349,9 +325,6 @@
     <t>TTR</t>
   </si>
   <si>
-    <t>NSCs</t>
-  </si>
-  <si>
     <t>+SOX2</t>
   </si>
   <si>
@@ -442,9 +415,6 @@
     <t>+PCP2</t>
   </si>
   <si>
-    <t>ChPCs</t>
-  </si>
-  <si>
     <t>+RGS5</t>
   </si>
   <si>
@@ -625,9 +595,6 @@
     <t xml:space="preserve">+RAB5A </t>
   </si>
   <si>
-    <t>OPCs</t>
-  </si>
-  <si>
     <t xml:space="preserve">+GPR17 </t>
   </si>
   <si>
@@ -734,6 +701,39 @@
   </si>
   <si>
     <t>PATH1R</t>
+  </si>
+  <si>
+    <t>OPC</t>
+  </si>
+  <si>
+    <t>Macrophage</t>
+  </si>
+  <si>
+    <t>Pericyte</t>
+  </si>
+  <si>
+    <t>Purkinje</t>
+  </si>
+  <si>
+    <t>Tanycyte</t>
+  </si>
+  <si>
+    <t>ChP</t>
+  </si>
+  <si>
+    <t>NSC</t>
+  </si>
+  <si>
+    <t>GPC</t>
+  </si>
+  <si>
+    <t>NPC</t>
+  </si>
+  <si>
+    <t>Astrocyte</t>
+  </si>
+  <si>
+    <t>Oligodendrocyte</t>
   </si>
 </sst>
 </file>
@@ -1086,122 +1086,122 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.88671875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="15.109375" style="1" customWidth="1"/>
-    <col min="19" max="20" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="16384" width="8.88671875" style="1"/>
+    <col min="15" max="15" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.85546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="15.140625" style="1" customWidth="1"/>
+    <col min="19" max="20" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>3</v>
+        <v>231</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>4</v>
+        <v>232</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>196</v>
+        <v>222</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>47</v>
+        <v>223</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>53</v>
+        <v>224</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>62</v>
+        <v>225</v>
       </c>
       <c r="R1" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="U1" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>135</v>
+        <v>227</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>104</v>
+        <v>228</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>100</v>
+        <v>229</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>99</v>
+        <v>230</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1209,245 +1209,245 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="G2" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q2" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="E4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="Z4" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I3" s="1" t="s">
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="E5" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E4" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E5" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>140</v>
-      </c>
       <c r="X5" s="1" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="J6" s="1" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="X6" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="Z6" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="X7" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="X8" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="Z8" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="X9" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z10" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="Z6" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="X7" s="1" t="s">
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z11" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="Z7" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="X8" s="1" t="s">
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z12" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="Z8" s="1" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="X9" s="1" t="s">
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="Z13" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="Z9" s="1" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="Z10" s="3" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="Z11" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="Z12" s="1" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="Z13" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="Z14" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="Z15" s="1" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -1460,448 +1460,448 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C011FA0D-996A-43C7-9FF4-C476D5920D18}">
   <dimension ref="A1:EC11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="8.88671875" style="4"/>
-    <col min="6" max="6" width="12.109375" style="4" customWidth="1"/>
-    <col min="7" max="29" width="8.88671875" style="4"/>
-    <col min="30" max="30" width="14.88671875" style="4" customWidth="1"/>
-    <col min="31" max="59" width="8.88671875" style="4"/>
-    <col min="60" max="60" width="14.88671875" style="4" customWidth="1"/>
-    <col min="61" max="64" width="8.88671875" style="4"/>
-    <col min="65" max="65" width="9.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="66" max="82" width="8.88671875" style="4"/>
-    <col min="83" max="83" width="11.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="84" max="16384" width="8.88671875" style="4"/>
+    <col min="1" max="5" width="8.85546875" style="4"/>
+    <col min="6" max="6" width="12.140625" style="4" customWidth="1"/>
+    <col min="7" max="29" width="8.85546875" style="4"/>
+    <col min="30" max="30" width="14.85546875" style="4" customWidth="1"/>
+    <col min="31" max="59" width="8.85546875" style="4"/>
+    <col min="60" max="60" width="14.85546875" style="4" customWidth="1"/>
+    <col min="61" max="64" width="8.85546875" style="4"/>
+    <col min="65" max="65" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="66" max="82" width="8.85546875" style="4"/>
+    <col min="83" max="83" width="11.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="84" max="16384" width="8.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:133" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:133" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="O1" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="P1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="AB1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AF1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG1" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="AH1" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="AI1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AL1" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="AM1" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="AN1" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="AP1" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="AQ1" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AR1" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="AS1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AT1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="AU1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="AV1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="AW1" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="AX1" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="AY1" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="AZ1" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="BA1" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="BB1" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="BC1" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="BD1" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="BE1" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="BF1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="BG1" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="BH1" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="BI1" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="BJ1" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="BK1" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="BL1" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="BM1" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="BN1" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="BO1" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="BP1" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="BQ1" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="BR1" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="BS1" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="P1" s="5" t="s">
+      <c r="BT1" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="BU1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="BV1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="BW1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="BX1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="BY1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="BZ1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="CA1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="CB1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="T1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="V1" s="5" t="s">
+      <c r="CC1" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="CD1" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="CE1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="CF1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="CG1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="CH1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="CI1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="CJ1" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="CK1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="CL1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="CM1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="CN1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="CO1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CP1" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="CQ1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="CR1" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="CS1" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="CT1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="CU1" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="CV1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="CW1" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="CX1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="CY1" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CZ1" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="DA1" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="DB1" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="DC1" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="DD1" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="DE1" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="DF1" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="W1" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="X1" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="Y1" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA1" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="AB1" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="AC1" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="AD1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="AE1" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="AF1" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="AG1" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="AH1" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="AI1" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AJ1" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="AK1" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="AL1" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="AM1" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="AN1" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="AO1" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="AP1" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AQ1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="AR1" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="AS1" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT1" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="AU1" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="AV1" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="AW1" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="AX1" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="AY1" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="AZ1" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="BA1" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="BB1" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="BC1" s="4" t="s">
+      <c r="DG1" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="DH1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="DI1" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="DJ1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="DK1" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="DL1" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="DM1" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="DN1" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="DO1" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="DP1" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="DQ1" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="DR1" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="DS1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="DT1" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="DU1" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="DV1" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="BD1" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="BE1" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="BF1" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="BG1" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="BH1" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="BI1" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="BJ1" s="4" t="s">
+      <c r="DW1" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="BK1" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="BL1" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="BM1" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="BN1" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="BO1" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="BP1" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="BQ1" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="BR1" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="BS1" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="BT1" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="BU1" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="BV1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="BW1" s="5" t="s">
+      <c r="DX1" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="DY1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="DZ1" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="EA1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="BX1" s="5" t="s">
+      <c r="EB1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="EC1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="BY1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="BZ1" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="CA1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="CB1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="CC1" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CD1" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="CE1" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="CF1" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="CG1" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="CH1" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="CI1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="CJ1" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="CK1" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="CL1" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="CM1" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="CN1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="CO1" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="CP1" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="CQ1" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="CR1" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="CS1" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="CT1" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="CU1" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="CV1" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="CW1" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="CX1" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="CY1" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="CZ1" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="DA1" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="DB1" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="DC1" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="DD1" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="DE1" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="DF1" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="DG1" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="DH1" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="DI1" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="DJ1" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="DK1" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="DL1" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="DM1" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="DN1" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="DO1" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="DP1" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="DQ1" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="DR1" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="DS1" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="DT1" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="DU1" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="DV1" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="DW1" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="DX1" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="DY1" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="DZ1" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="EA1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="EB1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="EC1" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:133" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:133" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:133" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:133" x14ac:dyDescent="0.25">
       <c r="CM6" s="1"/>
       <c r="CN6" s="1"/>
       <c r="CO6" s="1"/>
       <c r="CP6" s="1"/>
     </row>
-    <row r="7" spans="1:133" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:133" x14ac:dyDescent="0.25">
       <c r="CM7" s="1"/>
       <c r="CN7" s="1"/>
       <c r="CO7" s="1"/>
       <c r="CP7" s="1"/>
     </row>
-    <row r="8" spans="1:133" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:133" x14ac:dyDescent="0.25">
       <c r="CM8" s="1"/>
       <c r="CO8" s="1"/>
     </row>
-    <row r="9" spans="1:133" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:133" x14ac:dyDescent="0.25">
       <c r="CM9" s="1"/>
       <c r="CO9" s="1"/>
     </row>
-    <row r="10" spans="1:133" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:133" x14ac:dyDescent="0.25">
       <c r="CM10" s="1"/>
       <c r="CO10" s="1"/>
     </row>
-    <row r="11" spans="1:133" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:133" x14ac:dyDescent="0.25">
       <c r="CM11" s="1"/>
       <c r="CO11" s="1"/>
     </row>

</xml_diff>